<commit_message>
Add comprehensive peternakan data (hulu to hilir) with 7 sheets
</commit_message>
<xml_diff>
--- a/crypto_monitor.xlsx
+++ b/crypto_monitor.xlsx
@@ -479,7 +479,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W13"/>
+  <dimension ref="A1:W14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1477,6 +1477,80 @@
         <v>1.51</v>
       </c>
       <c r="V13" s="2" t="inlineStr">
+        <is>
+          <t>NETRAL ⚪</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>12:00</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="n">
+        <v>59836</v>
+      </c>
+      <c r="D14" s="3" t="n">
+        <v>1075026215</v>
+      </c>
+      <c r="E14" s="5" t="n">
+        <v>-1.56</v>
+      </c>
+      <c r="F14" s="3" t="n">
+        <v>1554.03</v>
+      </c>
+      <c r="G14" s="3" t="n">
+        <v>27919943</v>
+      </c>
+      <c r="H14" s="5" t="n">
+        <v>-3.88</v>
+      </c>
+      <c r="I14" s="3" t="n">
+        <v>68.04000000000001</v>
+      </c>
+      <c r="J14" s="3" t="n">
+        <v>1222333</v>
+      </c>
+      <c r="K14" s="4" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="L14" s="3" t="n">
+        <v>0.142268</v>
+      </c>
+      <c r="M14" s="3" t="n">
+        <v>2556</v>
+      </c>
+      <c r="N14" s="5" t="n">
+        <v>-3.29</v>
+      </c>
+      <c r="O14" s="3" t="n">
+        <v>0.074377</v>
+      </c>
+      <c r="P14" s="3" t="n">
+        <v>1336.27</v>
+      </c>
+      <c r="Q14" s="5" t="n">
+        <v>-2.02</v>
+      </c>
+      <c r="R14" s="3" t="n">
+        <v>1.03</v>
+      </c>
+      <c r="S14" s="3" t="n">
+        <v>18509.88</v>
+      </c>
+      <c r="T14" s="5" t="n">
+        <v>-3.63</v>
+      </c>
+      <c r="U14" s="6" t="n">
+        <v>1.51</v>
+      </c>
+      <c r="V14" s="2" t="inlineStr">
         <is>
           <t>NETRAL ⚪</t>
         </is>
@@ -1493,7 +1567,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G7"/>
+  <dimension ref="A1:G8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -1728,6 +1802,37 @@
         </is>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="B8" s="8" t="inlineStr">
+        <is>
+          <t>BTC</t>
+        </is>
+      </c>
+      <c r="C8" s="9" t="n">
+        <v>59836</v>
+      </c>
+      <c r="D8" s="12" t="n">
+        <v>-1.56</v>
+      </c>
+      <c r="E8" s="8" t="inlineStr">
+        <is>
+          <t>NETRAL</t>
+        </is>
+      </c>
+      <c r="F8" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="G8" s="11" t="inlineStr">
+        <is>
+          <t>Bitcoin Tembus Rp 1,9 M</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Fix crypto sheet name, update real prices from CoinGecko
</commit_message>
<xml_diff>
--- a/crypto_monitor.xlsx
+++ b/crypto_monitor.xlsx
@@ -7,7 +7,8 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Harga" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sentimen" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -34,8 +35,13 @@
       <b val="1"/>
       <color rgb="00FFFFFF"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -52,6 +58,24 @@
       <patternFill patternType="solid">
         <fgColor rgb="0010b981"/>
         <bgColor rgb="0010b981"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFCDD2"/>
+        <bgColor rgb="00FFCDD2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C8E6C9"/>
+        <bgColor rgb="00C8E6C9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001A237E"/>
+        <bgColor rgb="001A237E"/>
       </patternFill>
     </fill>
   </fills>
@@ -73,13 +97,43 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -445,8 +499,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V32"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:V33"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
@@ -2940,6 +2994,171 @@
         </is>
       </c>
     </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="B33" s="4" t="inlineStr">
+        <is>
+          <t>12:29</t>
+        </is>
+      </c>
+      <c r="C33" s="5" t="n">
+        <v>59878</v>
+      </c>
+      <c r="D33" s="5" t="n">
+        <v>1074710792</v>
+      </c>
+      <c r="E33" s="6" t="n">
+        <v>-1.51</v>
+      </c>
+      <c r="F33" s="5" t="n">
+        <v>1549.78</v>
+      </c>
+      <c r="G33" s="5" t="n">
+        <v>27815896</v>
+      </c>
+      <c r="H33" s="6" t="n">
+        <v>-4.14</v>
+      </c>
+      <c r="I33" s="5" t="n">
+        <v>67.98</v>
+      </c>
+      <c r="J33" s="5" t="n">
+        <v>1220102</v>
+      </c>
+      <c r="K33" s="7" t="n">
+        <v>0.64</v>
+      </c>
+      <c r="L33" s="5" t="n">
+        <v>0.142153</v>
+      </c>
+      <c r="M33" s="5" t="n">
+        <v>2551.4</v>
+      </c>
+      <c r="N33" s="6" t="n">
+        <v>-3.41</v>
+      </c>
+      <c r="O33" s="5" t="n">
+        <v>0.074281</v>
+      </c>
+      <c r="P33" s="5" t="n">
+        <v>1333.21</v>
+      </c>
+      <c r="Q33" s="6" t="n">
+        <v>-2.07</v>
+      </c>
+      <c r="R33" s="5" t="n">
+        <v>1.03</v>
+      </c>
+      <c r="S33" s="5" t="n">
+        <v>18479.55</v>
+      </c>
+      <c r="T33" s="6" t="n">
+        <v>-3.81</v>
+      </c>
+      <c r="U33" s="8" t="n">
+        <v>1.51</v>
+      </c>
+      <c r="V33" s="4" t="inlineStr">
+        <is>
+          <t>NETRAL ⚪</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <cols>
+    <col width="13" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="40" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="9" t="inlineStr">
+        <is>
+          <t>Tanggal</t>
+        </is>
+      </c>
+      <c r="B1" s="9" t="inlineStr">
+        <is>
+          <t>Koin</t>
+        </is>
+      </c>
+      <c r="C1" s="9" t="inlineStr">
+        <is>
+          <t>Harga (USD)</t>
+        </is>
+      </c>
+      <c r="D1" s="9" t="inlineStr">
+        <is>
+          <t>Perubahan 24h</t>
+        </is>
+      </c>
+      <c r="E1" s="9" t="inlineStr">
+        <is>
+          <t>Sentimen</t>
+        </is>
+      </c>
+      <c r="F1" s="9" t="inlineStr">
+        <is>
+          <t>Skor</t>
+        </is>
+      </c>
+      <c r="G1" s="9" t="inlineStr">
+        <is>
+          <t>Sumber Berita</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="10" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="B2" s="10" t="inlineStr">
+        <is>
+          <t>BTC</t>
+        </is>
+      </c>
+      <c r="C2" s="11" t="n">
+        <v>59878</v>
+      </c>
+      <c r="D2" s="12" t="n">
+        <v>-1.51</v>
+      </c>
+      <c r="E2" s="10" t="inlineStr">
+        <is>
+          <t>NETRAL</t>
+        </is>
+      </c>
+      <c r="F2" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="G2" s="13" t="inlineStr">
+        <is>
+          <t>Bitcoin Tembus Rp 1,9 M</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Fix column index - gas_elpiji should be row[17] not row[18]
</commit_message>
<xml_diff>
--- a/crypto_monitor.xlsx
+++ b/crypto_monitor.xlsx
@@ -499,8 +499,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V33"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <dimension ref="A1:V34"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
@@ -3068,6 +3068,80 @@
         </is>
       </c>
     </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="B34" s="4" t="inlineStr">
+        <is>
+          <t>18:00</t>
+        </is>
+      </c>
+      <c r="C34" s="5" t="n">
+        <v>59630</v>
+      </c>
+      <c r="D34" s="5" t="n">
+        <v>1063991608</v>
+      </c>
+      <c r="E34" s="6" t="n">
+        <v>-3.27</v>
+      </c>
+      <c r="F34" s="5" t="n">
+        <v>1550.6</v>
+      </c>
+      <c r="G34" s="5" t="n">
+        <v>27667890</v>
+      </c>
+      <c r="H34" s="6" t="n">
+        <v>-5.83</v>
+      </c>
+      <c r="I34" s="5" t="n">
+        <v>68.98</v>
+      </c>
+      <c r="J34" s="5" t="n">
+        <v>1230808</v>
+      </c>
+      <c r="K34" s="7" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="L34" s="5" t="n">
+        <v>0.143587</v>
+      </c>
+      <c r="M34" s="5" t="n">
+        <v>2562.07</v>
+      </c>
+      <c r="N34" s="6" t="n">
+        <v>-3.65</v>
+      </c>
+      <c r="O34" s="5" t="n">
+        <v>0.07394100000000001</v>
+      </c>
+      <c r="P34" s="5" t="n">
+        <v>1319.35</v>
+      </c>
+      <c r="Q34" s="6" t="n">
+        <v>-3.81</v>
+      </c>
+      <c r="R34" s="5" t="n">
+        <v>1.031</v>
+      </c>
+      <c r="S34" s="5" t="n">
+        <v>18394.14</v>
+      </c>
+      <c r="T34" s="6" t="n">
+        <v>-4.51</v>
+      </c>
+      <c r="U34" s="8" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="V34" s="4" t="inlineStr">
+        <is>
+          <t>NETRAL ⚪</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3079,8 +3153,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G2"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <dimension ref="A1:G3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
     <col width="8" customWidth="1" min="2" max="2"/>
@@ -3159,6 +3233,37 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" s="10" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="B3" s="10" t="inlineStr">
+        <is>
+          <t>BTC</t>
+        </is>
+      </c>
+      <c r="C3" s="11" t="n">
+        <v>59630</v>
+      </c>
+      <c r="D3" s="12" t="n">
+        <v>-3.27</v>
+      </c>
+      <c r="E3" s="10" t="inlineStr">
+        <is>
+          <t>NETRAL</t>
+        </is>
+      </c>
+      <c r="F3" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="G3" s="13" t="inlineStr">
+        <is>
+          <t>Bitcoin Tembus Rp 1,9 M</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Fix path issues in scripts: update_peternakan.py, update_saham.py, create_saham_ihsg.py
</commit_message>
<xml_diff>
--- a/crypto_monitor.xlsx
+++ b/crypto_monitor.xlsx
@@ -518,7 +518,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V2"/>
+  <dimension ref="A1:V3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -731,6 +731,80 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-27</t>
+        </is>
+      </c>
+      <c r="B3" s="8" t="inlineStr">
+        <is>
+          <t>17:45</t>
+        </is>
+      </c>
+      <c r="C3" s="9" t="n">
+        <v>60314</v>
+      </c>
+      <c r="D3" s="9" t="n">
+        <v>1077245809</v>
+      </c>
+      <c r="E3" s="10" t="n">
+        <v>0.89</v>
+      </c>
+      <c r="F3" s="9" t="n">
+        <v>1579.58</v>
+      </c>
+      <c r="G3" s="9" t="n">
+        <v>28212214</v>
+      </c>
+      <c r="H3" s="10" t="n">
+        <v>1.48</v>
+      </c>
+      <c r="I3" s="9" t="n">
+        <v>71.68000000000001</v>
+      </c>
+      <c r="J3" s="9" t="n">
+        <v>1280163</v>
+      </c>
+      <c r="K3" s="10" t="n">
+        <v>2.94</v>
+      </c>
+      <c r="L3" s="9" t="n">
+        <v>0.146803</v>
+      </c>
+      <c r="M3" s="9" t="n">
+        <v>2621.99</v>
+      </c>
+      <c r="N3" s="10" t="n">
+        <v>1.45</v>
+      </c>
+      <c r="O3" s="9" t="n">
+        <v>0.07522</v>
+      </c>
+      <c r="P3" s="9" t="n">
+        <v>1343.48</v>
+      </c>
+      <c r="Q3" s="10" t="n">
+        <v>1.16</v>
+      </c>
+      <c r="R3" s="9" t="n">
+        <v>1.055</v>
+      </c>
+      <c r="S3" s="9" t="n">
+        <v>18843.64</v>
+      </c>
+      <c r="T3" s="10" t="n">
+        <v>1.96</v>
+      </c>
+      <c r="U3" s="11" t="n">
+        <v>1.52</v>
+      </c>
+      <c r="V3" s="8" t="inlineStr">
+        <is>
+          <t>NETRAL ⚪</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -742,7 +816,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G2"/>
+  <dimension ref="A1:G3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -822,6 +896,37 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" s="12" t="inlineStr">
+        <is>
+          <t>2026-06-27</t>
+        </is>
+      </c>
+      <c r="B3" s="12" t="inlineStr">
+        <is>
+          <t>BTC</t>
+        </is>
+      </c>
+      <c r="C3" s="13" t="n">
+        <v>60314</v>
+      </c>
+      <c r="D3" s="14" t="n">
+        <v>0.89</v>
+      </c>
+      <c r="E3" s="12" t="inlineStr">
+        <is>
+          <t>NETRAL</t>
+        </is>
+      </c>
+      <c r="F3" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="G3" s="15" t="inlineStr">
+        <is>
+          <t>Bitcoin Tembus Rp 1,9 M</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>